<commit_message>
Add FastAPI backend routes for company search, detail, and facts
- Fix repository method placeholder bug found during live verification
- Expose GET /api/health, /api/companies/search, /api/companies/{id},
  /api/companies/{id}/facts
- Add .gitignore patterns for notebook checkpoints, R history, Excel lock files

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/reports/valuation/apple-day3-day4-model.xlsx
+++ b/docs/reports/valuation/apple-day3-day4-model.xlsx
@@ -250,6 +250,7 @@
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
   <chart>
     <title>
       <tx>
@@ -398,7 +399,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>11</row>
+      <row>14</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="6480000" cy="2880000"/>
@@ -8862,15 +8863,15 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>Complete-EV comps EV / EBITDA (AAPL + GOOGL)</t>
+          <t>Materiality-screened EV / EBITDA (AAPL + MSFT* + GOOGL)</t>
         </is>
       </c>
       <c r="B3" s="26">
-        <f>MIN('Comps'!Q2,'Comps'!Q4)</f>
+        <f>MIN('Comps'!Q2,'Comps'!Q3,'Comps'!Q4)</f>
         <v/>
       </c>
       <c r="C3" s="26">
-        <f>MAX('Comps'!Q2,'Comps'!Q4)</f>
+        <f>MAX('Comps'!Q2,'Comps'!Q3,'Comps'!Q4)</f>
         <v/>
       </c>
       <c r="D3" s="26">
@@ -8895,22 +8896,22 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Apple and Alphabet only: both EVs have complete identified debt and cash/investment inputs.</t>
+          <t>Apple and Alphabet complete; Microsoft re-included using stated FY2026 CommercialPaper = $0.000bn assumption based on FY2025.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>Complete-EV comps EV / Revenue (AAPL + GOOGL)</t>
+          <t>Materiality-screened EV / Revenue (AAPL + MSFT* + GOOGL)</t>
         </is>
       </c>
       <c r="B4" s="26">
-        <f>MIN('Comps'!R2,'Comps'!R4)</f>
+        <f>MIN('Comps'!R2,'Comps'!R3,'Comps'!R4)</f>
         <v/>
       </c>
       <c r="C4" s="26">
-        <f>MAX('Comps'!R2,'Comps'!R4)</f>
+        <f>MAX('Comps'!R2,'Comps'!R3,'Comps'!R4)</f>
         <v/>
       </c>
       <c r="D4" s="26">
@@ -8935,7 +8936,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Apple and Alphabet only: both EVs have complete identified debt and cash/investment inputs.</t>
+          <t>Apple and Alphabet complete; Microsoft re-included using stated FY2026 CommercialPaper = $0.000bn assumption based on FY2025.</t>
         </is>
       </c>
     </row>
@@ -9028,14 +9029,14 @@
       <c r="F7" s="17" t="n"/>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Excluded from EV-multiple implied-price ranges: MSFT, AMZN, META, NVDA, TSLA; details below. Exclusion is about EV completeness, not ingestion status.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="46" customHeight="1">
+          <t>* Microsoft re-included using a stated zero/near-zero assumption for CommercialPaper, based on the FY2025 value of $0.000bn at 2025-06-30. Amazon, Meta, NVIDIA, and Tesla remain excluded; see note below.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="68" customHeight="1">
       <c r="A8" s="27" t="inlineStr">
         <is>
-          <t>EV completeness screen: included AAPL and GOOGL (both database-ingested). Excluded MSFT, AMZN, and TSLA because commercial-paper facts were not found; excluded META because current debt and commercial paper were not found; excluded NVDA because FY2026 investments and commercial paper were not found. Missing amounts are unresolved, not zero. Provenance is separate: AMZN is database-ingested; MSFT, META, NVDA, and TSLA are capture-only. Ingestion status alone does not determine inclusion.</t>
+          <t>Materiality screen: Microsoft alone is re-included among previously excluded issuers, using FY2025 CommercialPaper of $0.000bn (2025-06-30) as an explicit assumption for missing FY2026 CommercialPaper, not a reported FY2026 fact. Amazon and Tesla CommercialPaper, and Meta current debt/commercial paper, have no adjacent low same-tag value; they remain excluded. NVIDIA FY2026 MarketableSecuritiesCurrent is missing; its FY2025 same-tag value was $34.621bn (2025-01-26), not low/near-zero, so NVIDIA remains excluded. This inclusion/exclusion rule is based on fact materiality, separately from ingestion status: Amazon is ingested but excluded; Microsoft is capture-only but re-included under assumption. NVIDIA and Meta remain excluded.</t>
         </is>
       </c>
     </row>

</xml_diff>